<commit_message>
test: update xlsx test fixture for multi-sheet e2e testing
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample-multisheet.xlsx
+++ b/tests/fixtures/sample-multisheet.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>名前</t>
   </si>
@@ -24,6 +24,9 @@
   </si>
   <si>
     <t>佐藤</t>
+  </si>
+  <si>
+    <t>部署名</t>
   </si>
   <si>
     <t>開発部</t>
@@ -88,6 +91,11 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>